<commit_message>
docs: update test plan with document information, objective, and scope
</commit_message>
<xml_diff>
--- a/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
+++ b/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f5fb949e079843e/Documents/GitHub/apache-fineract-manual-qa/02_Test_Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{8D5744B6-CF63-48B1-A2D5-9B9187E3967C}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{DEC11938-7826-471D-896A-FEDE040FB21A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,9 +53,6 @@
     <t>In Scope</t>
   </si>
   <si>
-    <t>Valid/Invalid Login, Validation, Logout, Session Timeout</t>
-  </si>
-  <si>
     <t>Out of Scope</t>
   </si>
   <si>
@@ -144,6 +141,16 @@
   </si>
   <si>
     <t>This test plan covers the manual functional testing of the Apache Fineract Login module, including user authentication, authorization, field validation, session management, logout functionality, and related security validations.</t>
+  </si>
+  <si>
+    <t>User Login - Verify login using valid credentials
+Invalid Login - Verify login using invalid credentials
+Mandatory Field Validation - Verify username and password are mandatory
+Password Masking - Verify password is hidden while typing
+User Authentication - Verify only authorized users can access the application
+Session Management - Verify user session timeout after inactivity
+Logout Functionality - Verify users can securely log out of the application
+Error Message Validation - Verify appropriate error messages are displayed for invalid login attempts</t>
   </si>
 </sst>
 </file>
@@ -294,15 +301,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -322,6 +323,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -629,181 +639,181 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" customWidth="1"/>
-    <col min="2" max="2" width="70" customWidth="1"/>
+    <col min="2" max="2" width="98.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="11"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="6">
+        <v>46236</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="3"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="8">
-        <v>46236</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" s="9" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14" s="9" t="s">
+    <row r="15" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" s="5" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="5" t="s">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="5" t="s">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="5" t="s">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="5" t="s">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="5" t="s">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="5" t="s">
+    </row>
+    <row r="22" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
+      <c r="B22" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update test plan with scope and project details
</commit_message>
<xml_diff>
--- a/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
+++ b/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f5fb949e079843e/Documents/GitHub/apache-fineract-manual-qa/02_Test_Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{8B2297E4-0282-42CF-87C4-C6F5EDD6896D}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{55736987-7D45-4E09-A467-C9185E98EE0F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,9 +56,6 @@
     <t>Out of Scope</t>
   </si>
   <si>
-    <t>Registration, Forgot Password, MFA</t>
-  </si>
-  <si>
     <t>Test Types</t>
   </si>
   <si>
@@ -151,6 +148,13 @@
 Session Management - Verify user session timeout after inactivity
 Logout Functionality - Verify users can securely log out of the application
 Error Message Validation - Verify appropriate error messages are displayed for invalid login attempts</t>
+  </si>
+  <si>
+    <t>User Registration - New user registration is not covered in this testing cycle
+Forgot Password - Password reset functionality is not included in this testing cycle
+Multi-Factor Authentication (MFA) - MFA functionality is not part of the current release
+User Profile Management - Profile update functionality is not included in this testing cycle
+Performance and Load Testing - Performance testing is excluded from the scope of this manual testing cycle</t>
   </si>
 </sst>
 </file>
@@ -324,14 +328,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -643,10 +647,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="11"/>
+      <c r="A1" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="12"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -682,55 +686,55 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B12" s="6">
         <v>46236</v>
@@ -741,7 +745,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -749,71 +753,71 @@
         <v>8</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>11</v>
+      <c r="B16" s="10" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update test plan with test strategy
</commit_message>
<xml_diff>
--- a/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
+++ b/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f5fb949e079843e/Documents/GitHub/apache-fineract-manual-qa/02_Test_Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{55736987-7D45-4E09-A467-C9185E98EE0F}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{E8156BE1-CDCE-401B-BC36-76AA459EC2EF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,9 +59,6 @@
     <t>Test Types</t>
   </si>
   <si>
-    <t>Smoke, Functional, Regression, System, UAT</t>
-  </si>
-  <si>
     <t>Entry Criteria</t>
   </si>
   <si>
@@ -155,6 +152,13 @@
 Multi-Factor Authentication (MFA) - MFA functionality is not part of the current release
 User Profile Management - Profile update functionality is not included in this testing cycle
 Performance and Load Testing - Performance testing is excluded from the scope of this manual testing cycle</t>
+  </si>
+  <si>
+    <t>Smoke Testing – Verify that the critical login functionality is working correctly before detailed testing begins.
+Functional Testing – Verify that all login features work according to the business requirements and functional specifications.
+Regression Testing – Verify that existing login functionality continues to work correctly after new changes, enhancements, or bug fixes.
+System Testing – Verify that the complete Login module functions correctly within the Apache Fineract application and integrates properly with related components.
+User Acceptance Testing (UAT) – Support business users in validating that the Login module meets business requirements and is ready for production use.</t>
   </si>
 </sst>
 </file>
@@ -305,7 +309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -336,6 +340,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -643,12 +650,12 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" customWidth="1"/>
-    <col min="2" max="2" width="98.85546875" customWidth="1"/>
+    <col min="2" max="2" width="111.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -686,55 +693,55 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>33</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12" s="6">
         <v>46236</v>
@@ -745,7 +752,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -753,7 +760,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -761,7 +768,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -769,55 +776,55 @@
         <v>10</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="10" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>21</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: add test environment to test plan
- Added application details
- Added QA environment
- Added browser information
- Added database details
- Added test data information
</commit_message>
<xml_diff>
--- a/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
+++ b/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f5fb949e079843e/Documents/GitHub/apache-fineract-manual-qa/02_Test_Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{E8156BE1-CDCE-401B-BC36-76AA459EC2EF}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{DECADE49-C697-4AC1-9A81-92A5E5B67B28}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Project Name</t>
   </si>
@@ -159,6 +159,16 @@
 Regression Testing – Verify that existing login functionality continues to work correctly after new changes, enhancements, or bug fixes.
 System Testing – Verify that the complete Login module functions correctly within the Apache Fineract application and integrates properly with related components.
 User Acceptance Testing (UAT) – Support business users in validating that the Login module meets business requirements and is ready for production use.</t>
+  </si>
+  <si>
+    <t>Test Environment</t>
+  </si>
+  <si>
+    <t>Application: Apache Fineract
+Environment: QA / Test Environment
+Browser: Google Chrome (Latest Stable Version)
+Database: MySQL
+Test Data: Dedicated QA test accounts and sample banking data</t>
   </si>
 </sst>
 </file>
@@ -646,7 +656,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" customWidth="1"/>
@@ -787,43 +797,51 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>13</v>
+    <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B22" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
+    <row r="23" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B23" s="9" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update test plan with entry criteria
- Added entry criteria
- Defined preconditions for test execution
</commit_message>
<xml_diff>
--- a/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
+++ b/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f5fb949e079843e/Documents/GitHub/apache-fineract-manual-qa/02_Test_Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{DECADE49-C697-4AC1-9A81-92A5E5B67B28}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{01C52E2B-E69D-496D-8B80-4F59CB2DB753}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,9 +62,6 @@
     <t>Entry Criteria</t>
   </si>
   <si>
-    <t>BRD approved, Test environment available</t>
-  </si>
-  <si>
     <t>Exit Criteria</t>
   </si>
   <si>
@@ -169,6 +166,13 @@
 Browser: Google Chrome (Latest Stable Version)
 Database: MySQL
 Test Data: Dedicated QA test accounts and sample banking data</t>
+  </si>
+  <si>
+    <t>Business Requirements Document (BRD) is reviewed and approved.
+Test environment is configured and accessible.
+A stable application build is available for testing.
+Required test data and test user accounts are available.
+All required access permissions are granted to the QA team.</t>
   </si>
 </sst>
 </file>
@@ -665,7 +669,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -703,55 +707,55 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" s="6">
         <v>46236</v>
@@ -762,7 +766,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -770,7 +774,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -778,7 +782,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -786,7 +790,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -794,55 +798,55 @@
         <v>11</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>13</v>
+      <c r="B19" s="10" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update test plan with exit criteria
</commit_message>
<xml_diff>
--- a/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
+++ b/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f5fb949e079843e/Documents/GitHub/apache-fineract-manual-qa/02_Test_Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{01C52E2B-E69D-496D-8B80-4F59CB2DB753}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{B92B613A-4B39-4E32-95C6-B742B68699CD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>Exit Criteria</t>
   </si>
   <si>
-    <t>All critical defects closed, test execution completed</t>
-  </si>
-  <si>
     <t>Deliverables</t>
   </si>
   <si>
@@ -173,6 +170,13 @@
 A stable application build is available for testing.
 Required test data and test user accounts are available.
 All required access permissions are granted to the QA team.</t>
+  </si>
+  <si>
+    <t>All planned test cases have been executed.
+All Critical and High severity defects are closed or accepted by stakeholders.
+No open Blocker defects remain.
+Test Summary Report is prepared and shared with stakeholders.
+Business stakeholders approve the application for release or provide formal sign-off for the completed testing cycle.</t>
   </si>
 </sst>
 </file>
@@ -669,7 +673,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -707,55 +711,55 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>21</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B12" s="6">
         <v>46236</v>
@@ -766,7 +770,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -774,7 +778,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -782,7 +786,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -790,7 +794,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -798,15 +802,15 @@
         <v>11</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>40</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -814,39 +818,39 @@
         <v>12</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>14</v>
+      <c r="B20" s="10" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>19</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: add test plan deliverables
- Added QA deliverables
- Defined project documentation outputs
</commit_message>
<xml_diff>
--- a/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
+++ b/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f5fb949e079843e/Documents/GitHub/apache-fineract-manual-qa/02_Test_Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{B92B613A-4B39-4E32-95C6-B742B68699CD}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{4684F12C-299B-4731-A3C1-8E6F4322221C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,9 +68,6 @@
     <t>Deliverables</t>
   </si>
   <si>
-    <t>Test Cases, Test Scenarios, Bug Report, RTM, Execution Report</t>
-  </si>
-  <si>
     <t>Risks</t>
   </si>
   <si>
@@ -177,6 +174,20 @@
 No open Blocker defects remain.
 Test Summary Report is prepared and shared with stakeholders.
 Business stakeholders approve the application for release or provide formal sign-off for the completed testing cycle.</t>
+  </si>
+  <si>
+    <t>Business Requirements Document (BRD)
+Test Plan
+Test Scenarios
+Test Cases
+Test Data
+Requirement Traceability Matrix (RTM)
+Bug / Defect Report
+Test Execution Report
+SQL Validation Scripts
+API Test Collection (Postman)
+Test Summary Report
+Release Sign-off Document</t>
   </si>
 </sst>
 </file>
@@ -673,7 +684,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B1" s="12"/>
     </row>
@@ -711,55 +722,55 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>20</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12" s="6">
         <v>46236</v>
@@ -770,7 +781,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -778,7 +789,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -786,7 +797,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -794,7 +805,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -802,15 +813,15 @@
         <v>11</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>39</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -818,7 +829,7 @@
         <v>12</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -826,31 +837,31 @@
         <v>13</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="345" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>15</v>
+      <c r="B21" s="10" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: add test plan assumptions
- Added project assumptions
- Documented testing dependencies
</commit_message>
<xml_diff>
--- a/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
+++ b/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f5fb949e079843e/Documents/GitHub/apache-fineract-manual-qa/02_Test_Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{4684F12C-299B-4731-A3C1-8E6F4322221C}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{2BC04741-2FFD-4520-A624-C0723DC5D85B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -71,13 +71,7 @@
     <t>Risks</t>
   </si>
   <si>
-    <t>Environment downtime, requirement changes</t>
-  </si>
-  <si>
     <t>Assumptions</t>
-  </si>
-  <si>
-    <t>Stable application and test environment</t>
   </si>
   <si>
     <t>Application Name</t>
@@ -188,6 +182,23 @@
 API Test Collection (Postman)
 Test Summary Report
 Release Sign-off Document</t>
+  </si>
+  <si>
+    <t>Requirement changes during the testing cycle.
+Test environment unavailability or instability.
+Delay in receiving application builds.
+Insufficient or incorrect test data.
+High-priority defects delaying test execution.
+Dependency on external systems or third-party services.
+Resource availability due to leave or workload.</t>
+  </si>
+  <si>
+    <t>Business requirements are complete and approved.
+The QA environment will remain available throughout testing.
+Valid test user accounts and test data are available.
+The application build provided for testing is stable.
+Required access to tools and environments is available.
+Stakeholders are available for requirement clarifications when needed.</t>
   </si>
 </sst>
 </file>
@@ -358,9 +369,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -372,6 +380,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -683,10 +694,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="12"/>
+      <c r="A1" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="11"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -722,55 +733,55 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B12" s="6">
         <v>46236</v>
@@ -781,7 +792,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -789,79 +800,79 @@
         <v>8</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>35</v>
+      <c r="B15" s="9" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="135" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="10" t="s">
+      <c r="B18" s="9" t="s">
         <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>40</v>
+      <c r="B19" s="9" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>41</v>
+      <c r="B20" s="9" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="345" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>18</v>
+      <c r="B23" s="13" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: complete Apache Fineract test plan v1.0
- Added roles and responsibilities
- Added test schedule
- Added approval section
- Completed Test Plan version 1.0
</commit_message>
<xml_diff>
--- a/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
+++ b/02_Test_Plan/Apache_Fineract_Test_Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8f5fb949e079843e/Documents/GitHub/apache-fineract-manual-qa/02_Test_Plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="85" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{2BC04741-2FFD-4520-A624-C0723DC5D85B}"/>
+  <xr:revisionPtr revIDLastSave="93" documentId="11_E94D148F576A487F601A04964CB306FF4B2389CD" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{877BE3FE-9C6A-4FA3-82F9-75E057A1DAF2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>Project Name</t>
   </si>
@@ -199,6 +199,68 @@
 The application build provided for testing is stable.
 Required access to tools and environments is available.
 Stakeholders are available for requirement clarifications when needed.</t>
+  </si>
+  <si>
+    <t>Roles &amp; Responsibilities</t>
+  </si>
+  <si>
+    <t>Business Analyst (BA)
+• Prepare and maintain business requirements.
+• Clarify functional requirements.
+QA Engineer
+• Analyze requirements.
+• Create test scenarios and test cases.
+• Execute test cases.
+• Report and verify defects.
+• Prepare test reports.
+Developer
+• Fix reported defects.
+• Support defect analysis.
+QA Lead
+• Review test artifacts.
+• Monitor testing progress.
+• Approve test deliverables.
+Project Manager
+• Monitor project timelines.
+• Coordinate between teams.
+• Approve project milestones.</t>
+  </si>
+  <si>
+    <t>Test Schedule</t>
+  </si>
+  <si>
+    <t>Requirement Analysis
+• Review Business Requirements Document (BRD).
+Test Planning
+• Prepare and review the Test Plan.
+Test Design
+• Create Test Scenarios and Test Cases.
+Test Data Preparation
+• Prepare test users and sample banking data.
+Test Execution
+• Execute planned test cases and record results.
+Defect Reporting
+• Log, track, and verify reported defects.
+Regression Testing
+• Re-test resolved defects and impacted functionality.
+Test Closure
+• Prepare the Test Summary Report and obtain sign-off.</t>
+  </si>
+  <si>
+    <t>Approval / Sign-off</t>
+  </si>
+  <si>
+    <t>Prepared By
+• Sachin Kodase
+• Manual QA Engineer
+Reviewed By
+• QA Lead
+• To Be Assigned (TBD)
+Approved By
+• Test Manager / Project Manager
+• To Be Assigned (TBD)
+Document Status
+• Draft (Version 1.0)</t>
   </si>
 </sst>
 </file>
@@ -247,7 +309,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -256,37 +318,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="thin">
@@ -300,90 +332,39 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -686,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" customWidth="1"/>
@@ -694,117 +675,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="11"/>
+      <c r="B1" s="2"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="7">
         <v>46236</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="8" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="120" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="9" t="s">
@@ -812,7 +793,7 @@
       </c>
     </row>
     <row r="16" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="9" t="s">
@@ -820,7 +801,7 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="135" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="10" t="s">
         <v>11</v>
       </c>
       <c r="B17" s="9" t="s">
@@ -828,7 +809,7 @@
       </c>
     </row>
     <row r="18" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="10" t="s">
         <v>36</v>
       </c>
       <c r="B18" s="9" t="s">
@@ -836,7 +817,7 @@
       </c>
     </row>
     <row r="19" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B19" s="9" t="s">
@@ -844,7 +825,7 @@
       </c>
     </row>
     <row r="20" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B20" s="9" t="s">
@@ -852,7 +833,7 @@
       </c>
     </row>
     <row r="21" spans="1:2" ht="345" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B21" s="9" t="s">
@@ -860,19 +841,43 @@
       </c>
     </row>
     <row r="22" spans="1:2" ht="195" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B22" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
+    <row r="23" spans="1:2" ht="165" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="9" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="360" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="345" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="210" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>